<commit_message>
talepler sayfası tekliflerle bağlandı.
</commit_message>
<xml_diff>
--- a/backend/app/temp/talep_listesi.xlsx
+++ b/backend/app/temp/talep_listesi.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t>SATINALMA TALEP LİSTESİ</t>
   </si>
   <si>
-    <t>Rapor Tarihi: 27.04.2026 19:35</t>
+    <t>Rapor Tarihi: 30.04.2026 14:48</t>
   </si>
   <si>
     <t>Sıra</t>
@@ -37,55 +37,151 @@
     <t>Birim</t>
   </si>
   <si>
+    <t>AA001</t>
+  </si>
+  <si>
+    <t>kurşun kalem</t>
+  </si>
+  <si>
+    <t>adet</t>
+  </si>
+  <si>
+    <t>a001</t>
+  </si>
+  <si>
+    <t>silgi</t>
+  </si>
+  <si>
+    <t>a002</t>
+  </si>
+  <si>
+    <t>defter</t>
+  </si>
+  <si>
     <t>PRD-0001</t>
   </si>
   <si>
-    <t>PVC elektrik borusu 20 mm</t>
+    <t>kalem turaş</t>
+  </si>
+  <si>
+    <t>a004</t>
+  </si>
+  <si>
+    <t>pergel</t>
+  </si>
+  <si>
+    <t>a005</t>
+  </si>
+  <si>
+    <t>cetvel</t>
+  </si>
+  <si>
+    <t>a003</t>
+  </si>
+  <si>
+    <t>kalem tıraş</t>
+  </si>
+  <si>
+    <t>a006</t>
+  </si>
+  <si>
+    <t>kalem</t>
+  </si>
+  <si>
+    <t>PRD-0002</t>
+  </si>
+  <si>
+    <t>PİLOT KALEM</t>
+  </si>
+  <si>
+    <t>A102</t>
+  </si>
+  <si>
+    <t>SİLGİ BÜYÜK</t>
+  </si>
+  <si>
+    <t>A104</t>
+  </si>
+  <si>
+    <t>DOSYA KLASÖR</t>
+  </si>
+  <si>
+    <t>A105</t>
+  </si>
+  <si>
+    <t>ZIMBA MAKİNESİ</t>
+  </si>
+  <si>
+    <t>PRD-0003</t>
+  </si>
+  <si>
+    <t>Ahşap ve hafif metal montajı için uygun, galvaniz kaplı</t>
+  </si>
+  <si>
+    <t>PRD-0004</t>
+  </si>
+  <si>
+    <t>İç tesisat kablo geçişi için</t>
   </si>
   <si>
     <t>metre</t>
   </si>
   <si>
-    <t>PRD-0002</t>
-  </si>
-  <si>
-    <t>Kablo bağı 200x3.6 mm</t>
-  </si>
-  <si>
-    <t>adet</t>
-  </si>
-  <si>
-    <t>PRD-0003</t>
-  </si>
-  <si>
-    <t>Lateks eldiven</t>
+    <t>PRD-0005</t>
+  </si>
+  <si>
+    <t>Siyah, UV dayanımlı</t>
+  </si>
+  <si>
+    <t>PRD-0006</t>
+  </si>
+  <si>
+    <t>Tek kullanımlık, pudrasız</t>
   </si>
   <si>
     <t>kutu</t>
   </si>
   <si>
-    <t>PRD-0004</t>
-  </si>
-  <si>
-    <t>Akrilik mastik beyaz</t>
-  </si>
-  <si>
-    <t>PRD-0005</t>
-  </si>
-  <si>
-    <t>Spiral taşlama diski 115 mm</t>
-  </si>
-  <si>
-    <t>PRD-0006</t>
-  </si>
-  <si>
-    <t>İzolasyon bandı siyah</t>
-  </si>
-  <si>
     <t>PRD-0007</t>
   </si>
   <si>
-    <t>Temizlik bezi mikrofiber</t>
+    <t>İç cephe boşluk doldurma uygulaması</t>
+  </si>
+  <si>
+    <t>PRD-0008</t>
+  </si>
+  <si>
+    <t>Metal kesim için</t>
+  </si>
+  <si>
+    <t>PRD-0009</t>
+  </si>
+  <si>
+    <t>Elektrik bağlantı izolasyonu</t>
+  </si>
+  <si>
+    <t>PRD-0010</t>
+  </si>
+  <si>
+    <t>Genel yüzey temizliği için</t>
+  </si>
+  <si>
+    <t>A101</t>
+  </si>
+  <si>
+    <t>PİLOT KALEM MAVİ</t>
+  </si>
+  <si>
+    <t>A103</t>
+  </si>
+  <si>
+    <t>DEFTER A4</t>
+  </si>
+  <si>
+    <t>PRD-0011</t>
+  </si>
+  <si>
+    <t>uçlu kalem</t>
   </si>
 </sst>
 </file>
@@ -464,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -512,7 +608,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="3">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>9</v>
@@ -529,10 +625,10 @@
         <v>11</v>
       </c>
       <c r="D7" s="3">
-        <v>500</v>
+        <v>110</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -540,16 +636,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>14</v>
-      </c>
       <c r="D8" s="3">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -557,16 +653,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" s="3">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -574,16 +670,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D10" s="3">
-        <v>40</v>
+        <v>260</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -591,16 +687,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D11" s="3">
-        <v>75</v>
+        <v>210</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -608,16 +704,288 @@
         <v>7</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="3">
+        <v>120</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="3">
+        <v>8</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D13" s="3">
+        <v>5</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="3">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3">
+        <v>90</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="3">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="3">
+        <v>275</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="3">
+        <v>11</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="3">
+        <v>60</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="3">
+        <v>12</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>12</v>
+      <c r="C17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="3">
+        <v>40</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="3">
+        <v>13</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="3">
+        <v>250</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="3">
+        <v>14</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="3">
+        <v>120</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="3">
+        <v>15</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="3">
+        <v>500</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="3">
+        <v>16</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="3">
+        <v>20</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="3">
+        <v>17</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="3">
+        <v>36</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="3">
+        <v>18</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="3">
+        <v>40</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="3">
+        <v>19</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" s="3">
+        <v>75</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="3">
+        <v>20</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="3">
+        <v>30</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="3">
+        <v>21</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="3">
+        <v>410</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="3">
+        <v>22</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D27" s="3">
+        <v>150</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="3">
+        <v>23</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="3">
+        <v>70</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
teklifler excel ve pdf okuyor ve doğru rapor veriyor.
</commit_message>
<xml_diff>
--- a/backend/app/temp/talep_listesi.xlsx
+++ b/backend/app/temp/talep_listesi.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
   <si>
     <t>SATINALMA TALEP LİSTESİ</t>
   </si>
   <si>
-    <t>Rapor Tarihi: 30.04.2026 14:48</t>
+    <t>Rapor Tarihi: 04.05.2026 20:34</t>
   </si>
   <si>
     <t>Sıra</t>
@@ -37,148 +37,88 @@
     <t>Birim</t>
   </si>
   <si>
+    <t>A101</t>
+  </si>
+  <si>
+    <t>PİLOT KALEM MAVİ</t>
+  </si>
+  <si>
+    <t>adet</t>
+  </si>
+  <si>
+    <t>A102</t>
+  </si>
+  <si>
+    <t>SİLGİ BÜYÜK</t>
+  </si>
+  <si>
+    <t>A103</t>
+  </si>
+  <si>
+    <t>DEFTER A4</t>
+  </si>
+  <si>
+    <t>a004</t>
+  </si>
+  <si>
+    <t>PERGEL</t>
+  </si>
+  <si>
+    <t>a005</t>
+  </si>
+  <si>
+    <t>CETVEL</t>
+  </si>
+  <si>
+    <t>PRD-0001</t>
+  </si>
+  <si>
+    <t>PİLOT KALEM</t>
+  </si>
+  <si>
+    <t>A104</t>
+  </si>
+  <si>
+    <t>DOSYA KLASÖR</t>
+  </si>
+  <si>
+    <t>A105</t>
+  </si>
+  <si>
+    <t>ZIMBA MAKİNESİ</t>
+  </si>
+  <si>
+    <t>a001</t>
+  </si>
+  <si>
+    <t>silgi</t>
+  </si>
+  <si>
+    <t>a002</t>
+  </si>
+  <si>
+    <t>defter</t>
+  </si>
+  <si>
+    <t>a003</t>
+  </si>
+  <si>
+    <t>kalem tıraş</t>
+  </si>
+  <si>
+    <t>a006</t>
+  </si>
+  <si>
+    <t>kalem</t>
+  </si>
+  <si>
     <t>AA001</t>
   </si>
   <si>
     <t>kurşun kalem</t>
   </si>
   <si>
-    <t>adet</t>
-  </si>
-  <si>
-    <t>a001</t>
-  </si>
-  <si>
-    <t>silgi</t>
-  </si>
-  <si>
-    <t>a002</t>
-  </si>
-  <si>
-    <t>defter</t>
-  </si>
-  <si>
-    <t>PRD-0001</t>
-  </si>
-  <si>
-    <t>kalem turaş</t>
-  </si>
-  <si>
-    <t>a004</t>
-  </si>
-  <si>
-    <t>pergel</t>
-  </si>
-  <si>
-    <t>a005</t>
-  </si>
-  <si>
-    <t>cetvel</t>
-  </si>
-  <si>
-    <t>a003</t>
-  </si>
-  <si>
-    <t>kalem tıraş</t>
-  </si>
-  <si>
-    <t>a006</t>
-  </si>
-  <si>
-    <t>kalem</t>
-  </si>
-  <si>
     <t>PRD-0002</t>
-  </si>
-  <si>
-    <t>PİLOT KALEM</t>
-  </si>
-  <si>
-    <t>A102</t>
-  </si>
-  <si>
-    <t>SİLGİ BÜYÜK</t>
-  </si>
-  <si>
-    <t>A104</t>
-  </si>
-  <si>
-    <t>DOSYA KLASÖR</t>
-  </si>
-  <si>
-    <t>A105</t>
-  </si>
-  <si>
-    <t>ZIMBA MAKİNESİ</t>
-  </si>
-  <si>
-    <t>PRD-0003</t>
-  </si>
-  <si>
-    <t>Ahşap ve hafif metal montajı için uygun, galvaniz kaplı</t>
-  </si>
-  <si>
-    <t>PRD-0004</t>
-  </si>
-  <si>
-    <t>İç tesisat kablo geçişi için</t>
-  </si>
-  <si>
-    <t>metre</t>
-  </si>
-  <si>
-    <t>PRD-0005</t>
-  </si>
-  <si>
-    <t>Siyah, UV dayanımlı</t>
-  </si>
-  <si>
-    <t>PRD-0006</t>
-  </si>
-  <si>
-    <t>Tek kullanımlık, pudrasız</t>
-  </si>
-  <si>
-    <t>kutu</t>
-  </si>
-  <si>
-    <t>PRD-0007</t>
-  </si>
-  <si>
-    <t>İç cephe boşluk doldurma uygulaması</t>
-  </si>
-  <si>
-    <t>PRD-0008</t>
-  </si>
-  <si>
-    <t>Metal kesim için</t>
-  </si>
-  <si>
-    <t>PRD-0009</t>
-  </si>
-  <si>
-    <t>Elektrik bağlantı izolasyonu</t>
-  </si>
-  <si>
-    <t>PRD-0010</t>
-  </si>
-  <si>
-    <t>Genel yüzey temizliği için</t>
-  </si>
-  <si>
-    <t>A101</t>
-  </si>
-  <si>
-    <t>PİLOT KALEM MAVİ</t>
-  </si>
-  <si>
-    <t>A103</t>
-  </si>
-  <si>
-    <t>DEFTER A4</t>
-  </si>
-  <si>
-    <t>PRD-0011</t>
   </si>
   <si>
     <t>uçlu kalem</t>
@@ -560,7 +500,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
@@ -608,7 +548,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="3">
-        <v>50</v>
+        <v>410</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>9</v>
@@ -625,7 +565,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="3">
-        <v>110</v>
+        <v>275</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>9</v>
@@ -642,7 +582,7 @@
         <v>13</v>
       </c>
       <c r="D8" s="3">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>9</v>
@@ -659,7 +599,7 @@
         <v>15</v>
       </c>
       <c r="D9" s="3">
-        <v>40</v>
+        <v>260</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>9</v>
@@ -676,7 +616,7 @@
         <v>17</v>
       </c>
       <c r="D10" s="3">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>9</v>
@@ -693,7 +633,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="3">
-        <v>210</v>
+        <v>90</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>9</v>
@@ -710,7 +650,7 @@
         <v>21</v>
       </c>
       <c r="D12" s="3">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>9</v>
@@ -727,7 +667,7 @@
         <v>23</v>
       </c>
       <c r="D13" s="3">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>9</v>
@@ -744,7 +684,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="3">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>9</v>
@@ -761,7 +701,7 @@
         <v>27</v>
       </c>
       <c r="D15" s="3">
-        <v>275</v>
+        <v>110</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>9</v>
@@ -778,7 +718,7 @@
         <v>29</v>
       </c>
       <c r="D16" s="3">
-        <v>60</v>
+        <v>160</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>9</v>
@@ -795,7 +735,7 @@
         <v>31</v>
       </c>
       <c r="D17" s="3">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>9</v>
@@ -812,7 +752,7 @@
         <v>33</v>
       </c>
       <c r="D18" s="3">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>9</v>
@@ -829,162 +769,9 @@
         <v>35</v>
       </c>
       <c r="D19" s="3">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="3">
-        <v>15</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D20" s="3">
-        <v>500</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="3">
-        <v>16</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="3">
-        <v>20</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="3">
-        <v>17</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D22" s="3">
-        <v>36</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="3">
-        <v>18</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D23" s="3">
-        <v>40</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="3">
-        <v>19</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="3">
-        <v>75</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="3">
-        <v>20</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" s="3">
-        <v>30</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="3">
-        <v>21</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26" s="3">
-        <v>410</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="3">
-        <v>22</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27" s="3">
-        <v>150</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="3">
-        <v>23</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28" s="3">
-        <v>70</v>
-      </c>
-      <c r="E28" s="3" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>